<commit_message>
Complete Sprint 6 deliverables
</commit_message>
<xml_diff>
--- a/output/company_clusters.xlsx
+++ b/output/company_clusters.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>distance_from_centroid</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>cluster_name</t>
         </is>
       </c>
@@ -508,11 +513,14 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.2018</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -551,11 +559,14 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.3404</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -594,11 +605,14 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.2663</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -639,7 +653,10 @@
       <c r="J5" t="n">
         <v>2</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" t="n">
+        <v>2.3837</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -681,11 +698,14 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.1831</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -726,7 +746,10 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="n">
+        <v>0.8085</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -767,11 +790,14 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.0059</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -811,11 +837,14 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.5694</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -855,11 +884,14 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.0197</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -896,11 +928,14 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.2507</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -941,7 +976,10 @@
       <c r="J12" t="n">
         <v>2</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K12" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -982,11 +1020,14 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.8198</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1068,10 @@
       <c r="J14" t="n">
         <v>2</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" t="n">
+        <v>0.9962</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -1068,11 +1112,14 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2.1447</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1160,10 @@
       <c r="J16" t="n">
         <v>2</v>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K16" t="n">
+        <v>1.3882</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -1156,7 +1206,10 @@
       <c r="J17" t="n">
         <v>2</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" t="n">
+        <v>1.7064</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -1197,11 +1250,14 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.8711</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1240,11 +1296,14 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1.4412</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -1284,11 +1343,14 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2.1803</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1327,11 +1389,14 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.6261</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1437,10 @@
       <c r="J22" t="n">
         <v>0</v>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" t="n">
+        <v>1.6009</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -1415,7 +1483,10 @@
       <c r="J23" t="n">
         <v>0</v>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" t="n">
+        <v>0.5017</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -1458,7 +1529,10 @@
       <c r="J24" t="n">
         <v>2</v>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K24" t="n">
+        <v>2.8937</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -1501,7 +1575,10 @@
       <c r="J25" t="n">
         <v>2</v>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -1543,11 +1620,14 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.7305</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1668,10 @@
       <c r="J27" t="n">
         <v>0</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" t="n">
+        <v>1.9791</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -1629,11 +1712,14 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.7655999999999999</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1672,11 +1758,14 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1715,11 +1804,14 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>2.1618</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1758,11 +1850,14 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.4568</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1801,11 +1896,14 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.6476</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1844,11 +1942,14 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.5993000000000001</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1887,11 +1988,14 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1930,11 +2034,14 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1.1011</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -1973,11 +2080,14 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.6513</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2016,11 +2126,14 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.9366</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2059,11 +2172,14 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1.103</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2102,11 +2218,14 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.5862000000000001</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2266,10 @@
       <c r="J40" t="n">
         <v>2</v>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" t="n">
+        <v>0.7413</v>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -2188,11 +2310,14 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.7003</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2232,11 +2357,14 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.7739</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2275,11 +2403,14 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.7298</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2319,11 +2450,14 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.7613</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2498,10 @@
       <c r="J45" t="n">
         <v>2</v>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" t="n">
+        <v>1.165</v>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -2405,11 +2542,14 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>1</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.6963</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2448,11 +2588,14 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.0092</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2491,11 +2634,14 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>1</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.7194</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2682,10 @@
       <c r="J49" t="n">
         <v>2</v>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" t="n">
+        <v>0.8625</v>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -2577,11 +2726,14 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1.0662</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2621,11 +2773,14 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1.7686</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2821,10 @@
       <c r="J52" t="n">
         <v>0</v>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K52" t="n">
+        <v>1.6294</v>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -2709,7 +2867,10 @@
       <c r="J53" t="n">
         <v>2</v>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K53" t="n">
+        <v>2.2405</v>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -2751,11 +2912,14 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1.2571</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2794,11 +2958,14 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1.8768</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2837,11 +3004,14 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>1</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.9839</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -2880,11 +3050,14 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1.3851</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2923,11 +3096,14 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1.4104</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -2967,11 +3143,14 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K59" t="n">
+        <v>2.2386</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3191,10 @@
       <c r="J60" t="n">
         <v>0</v>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="K60" t="n">
+        <v>0.9468</v>
+      </c>
+      <c r="L60" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -3053,11 +3235,14 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K61" t="n">
+        <v>1.6693</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3096,11 +3281,14 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3139,11 +3327,14 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K63" t="n">
+        <v>2.5981</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3183,11 +3374,14 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.7205</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3226,11 +3420,14 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.4664</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3269,11 +3466,14 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.6113</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3312,11 +3512,14 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1.1948</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3560,10 @@
       <c r="J68" t="n">
         <v>0</v>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="K68" t="n">
+        <v>4.5331</v>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -3399,11 +3605,14 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K69" t="n">
+        <v>1.6449</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3442,11 +3651,14 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.5038</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3485,11 +3697,14 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.6195000000000001</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3745,10 @@
       <c r="J72" t="n">
         <v>2</v>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="K72" t="n">
+        <v>1.4161</v>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -3571,11 +3789,14 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.8058</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3614,11 +3835,14 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K74" t="n">
+        <v>1.2971</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3657,11 +3881,14 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K75" t="n">
+        <v>1.2935</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -3700,11 +3927,14 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>1</v>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>High Growth</t>
+        <v>3</v>
+      </c>
+      <c r="K76" t="n">
+        <v>1.999</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Turnaround / Risk</t>
         </is>
       </c>
     </row>
@@ -3744,11 +3974,14 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1.0096</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3787,11 +4020,14 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>0</v>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1.7953</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3828,11 +4064,14 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>0</v>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1.4032</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3871,11 +4110,14 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>0</v>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.4829</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -3917,7 +4159,10 @@
       <c r="J81" t="n">
         <v>2</v>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="K81" t="n">
+        <v>1.3659</v>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -3958,11 +4203,14 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.7577</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4001,11 +4249,14 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1.5882</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4044,11 +4295,14 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>0</v>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K84" t="n">
+        <v>2.6425</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4343,10 @@
       <c r="J85" t="n">
         <v>0</v>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="K85" t="n">
+        <v>1.2835</v>
+      </c>
+      <c r="L85" t="inlineStr">
         <is>
           <t>Stable Compounders</t>
         </is>
@@ -4131,11 +4388,14 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>0</v>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4175,11 +4435,14 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>0</v>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4218,11 +4481,14 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1.0804</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4261,11 +4527,14 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.9101</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4305,11 +4574,14 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>0</v>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K90" t="n">
+        <v>1.7663</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4348,11 +4620,14 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.8212</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4391,11 +4666,14 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>3</v>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>Turnaround / Risk</t>
+        <v>4</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Defensive</t>
         </is>
       </c>
     </row>
@@ -4434,11 +4712,14 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>0</v>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K93" t="n">
+        <v>1.1955</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4473,11 +4754,14 @@
       </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="n">
-        <v>0</v>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0.2682</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4798,10 @@
       <c r="J95" t="n">
         <v>2</v>
       </c>
-      <c r="K95" t="inlineStr">
+      <c r="K95" t="n">
+        <v>2.3532</v>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -4549,11 +4836,14 @@
       </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="n">
-        <v>0</v>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K96" t="n">
+        <v>1.1624</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4586,11 +4876,14 @@
       </c>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="n">
-        <v>0</v>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K97" t="n">
+        <v>1.7737</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4623,11 +4916,14 @@
       </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="n">
-        <v>0</v>
-      </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4660,11 +4956,14 @@
       </c>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="n">
-        <v>0</v>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0.5615</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4998,10 @@
       <c r="J100" t="n">
         <v>2</v>
       </c>
-      <c r="K100" t="inlineStr">
+      <c r="K100" t="n">
+        <v>4.6671</v>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>Value Picks</t>
         </is>
@@ -4734,11 +5036,14 @@
       </c>
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="n">
-        <v>0</v>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>Stable Compounders</t>
+        <v>1</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0.4627</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>High Growth</t>
         </is>
       </c>
     </row>

</xml_diff>